<commit_message>
test: expand coverage for service, ingestion, and mailbox flows
- add unit coverage for mapping, parsing, FIX, reporting, dashboard, mailbox, service, and ingestion behaviors
- add interface seams for email, parser, FIX engine, and FIX client to support isolated testing
- update FixFlowService and FixFlowWeb composition to use the new abstractions
- harden side normalization with regression coverage for enum parsing
- remove legacy Weather page and clean up old attachment samples
</commit_message>
<xml_diff>
--- a/attachments/Allocations_Multiple.xlsx
+++ b/attachments/Allocations_Multiple.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zakme\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Apps\FixFlow.TradeAllocBridge\attachments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341EF895-3610-4B49-B6DA-FF8CD2A87492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C5C32D-07D0-4C87-B354-8E8FB5B5A9D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="24792" windowHeight="13320" xr2:uid="{619E463A-8D35-493B-A9CF-06F38D4871CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{619E463A-8D35-493B-A9CF-06F38D4871CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Allocations_Multiple" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="24">
   <si>
     <t xml:space="preserve">Cust </t>
   </si>
@@ -46,15 +46,9 @@
     <t xml:space="preserve">SettleDate </t>
   </si>
   <si>
-    <t>Route</t>
-  </si>
-  <si>
     <t>GS</t>
   </si>
   <si>
-    <t>RAJA</t>
-  </si>
-  <si>
     <t>Buy</t>
   </si>
   <si>
@@ -64,9 +58,6 @@
     <t>USD</t>
   </si>
   <si>
-    <t>RAJA-CARE-US</t>
-  </si>
-  <si>
     <t>MSCO</t>
   </si>
   <si>
@@ -95,6 +86,12 @@
   </si>
   <si>
     <t>Sell</t>
+  </si>
+  <si>
+    <t>BROK</t>
+  </si>
+  <si>
+    <t>BOFA</t>
   </si>
 </sst>
 </file>
@@ -964,17 +961,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{844F7F59-E9C6-4A76-90C6-EE6F204EE0B8}">
-  <dimension ref="A1:N19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="5" max="5" width="10.88671875" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" customWidth="1"/>
-    <col min="12" max="12" width="11.109375" customWidth="1"/>
-    <col min="13" max="13" width="11.21875" customWidth="1"/>
+    <col min="5" max="5" width="10.89453125" customWidth="1"/>
+    <col min="8" max="8" width="12.89453125" customWidth="1"/>
+    <col min="9" max="9" width="13.5234375" customWidth="1"/>
+    <col min="12" max="12" width="11.1015625" customWidth="1"/>
+    <col min="13" max="13" width="11.20703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -982,16 +979,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G1" t="s">
         <v>2</v>
@@ -1009,27 +1006,24 @@
         <v>6</v>
       </c>
       <c r="L1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="N1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
       </c>
       <c r="E2" s="1">
         <v>9797</v>
@@ -1038,7 +1032,7 @@
         <v>61.370399999999997</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H2" s="2">
         <v>601245.81000000006</v>
@@ -1058,22 +1052,19 @@
       <c r="M2" s="3">
         <v>45960</v>
       </c>
-      <c r="N2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
       </c>
       <c r="E3" s="1">
         <v>12319</v>
@@ -1082,7 +1073,7 @@
         <v>61.370399999999997</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H3" s="2">
         <v>756021.96</v>
@@ -1102,22 +1093,19 @@
       <c r="M3" s="3">
         <v>45960</v>
       </c>
-      <c r="N3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
       </c>
       <c r="E4" s="1">
         <v>1810</v>
@@ -1126,7 +1114,7 @@
         <v>61.370399999999997</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H4" s="2">
         <v>111080.42</v>
@@ -1146,22 +1134,19 @@
       <c r="M4" s="3">
         <v>45960</v>
       </c>
-      <c r="N4" t="s">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
       <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
         <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
       </c>
       <c r="E5" s="1">
         <v>1074</v>
@@ -1170,7 +1155,7 @@
         <v>61.370399999999997</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H5" s="2">
         <v>65911.81</v>
@@ -1190,22 +1175,19 @@
       <c r="M5" s="3">
         <v>45960</v>
       </c>
-      <c r="N5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
       </c>
       <c r="E6" s="1">
         <v>9805</v>
@@ -1214,7 +1196,7 @@
         <v>60.504300000000001</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H6" s="2">
         <v>593244.66</v>
@@ -1234,22 +1216,19 @@
       <c r="M6" s="3">
         <v>45960</v>
       </c>
-      <c r="N6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
         <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
       </c>
       <c r="E7" s="1">
         <v>12315</v>
@@ -1258,7 +1237,7 @@
         <v>60.504300000000001</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H7" s="2">
         <v>745110.45</v>
@@ -1278,22 +1257,19 @@
       <c r="M7" s="3">
         <v>45960</v>
       </c>
-      <c r="N7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
         <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
       </c>
       <c r="E8" s="1">
         <v>1806</v>
@@ -1302,7 +1278,7 @@
         <v>60.504300000000001</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H8" s="2">
         <v>109270.77</v>
@@ -1322,22 +1298,19 @@
       <c r="M8" s="3">
         <v>45960</v>
       </c>
-      <c r="N8" t="s">
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
       <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
         <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
       </c>
       <c r="E9" s="1">
         <v>1074</v>
@@ -1346,7 +1319,7 @@
         <v>60.504300000000001</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H9" s="2">
         <v>64981.62</v>
@@ -1366,22 +1339,19 @@
       <c r="M9" s="3">
         <v>45960</v>
       </c>
-      <c r="N9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
         <v>10</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
       </c>
       <c r="E10" s="1">
         <v>9784</v>
@@ -1390,7 +1360,7 @@
         <v>60.696899999999999</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H10" s="2">
         <v>593858.47</v>
@@ -1410,22 +1380,19 @@
       <c r="M10" s="3">
         <v>45960</v>
       </c>
-      <c r="N10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
         <v>10</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" t="s">
-        <v>12</v>
       </c>
       <c r="E11" s="1">
         <v>12326</v>
@@ -1434,7 +1401,7 @@
         <v>60.696899999999999</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H11" s="2">
         <v>748149.99</v>
@@ -1454,22 +1421,19 @@
       <c r="M11" s="3">
         <v>45960</v>
       </c>
-      <c r="N11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
         <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
       </c>
       <c r="E12" s="1">
         <v>1814</v>
@@ -1478,7 +1442,7 @@
         <v>60.696899999999999</v>
       </c>
       <c r="G12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H12" s="2">
         <v>110104.18</v>
@@ -1498,22 +1462,19 @@
       <c r="M12" s="3">
         <v>45960</v>
       </c>
-      <c r="N12" t="s">
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>17</v>
-      </c>
       <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
         <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
       </c>
       <c r="E13" s="1">
         <v>1076</v>
@@ -1522,7 +1483,7 @@
         <v>60.696899999999999</v>
       </c>
       <c r="G13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H13" s="2">
         <v>65309.86</v>
@@ -1542,22 +1503,19 @@
       <c r="M13" s="3">
         <v>45960</v>
       </c>
-      <c r="N13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s">
         <v>15</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" t="s">
-        <v>18</v>
       </c>
       <c r="E14" s="1">
         <v>1200</v>
@@ -1566,7 +1524,7 @@
         <v>44.499600000000001</v>
       </c>
       <c r="G14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H14" s="2">
         <v>53399.519999999997</v>
@@ -1586,22 +1544,19 @@
       <c r="M14" s="3">
         <v>45960</v>
       </c>
-      <c r="N14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
         <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" t="s">
-        <v>12</v>
       </c>
       <c r="E15" s="1">
         <v>4717</v>
@@ -1610,7 +1565,7 @@
         <v>60.944699999999997</v>
       </c>
       <c r="G15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H15" s="2">
         <v>287476.15000000002</v>
@@ -1630,22 +1585,19 @@
       <c r="M15" s="3">
         <v>45960</v>
       </c>
-      <c r="N15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
         <v>10</v>
-      </c>
-      <c r="C16" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" t="s">
-        <v>12</v>
       </c>
       <c r="E16" s="1">
         <v>5943</v>
@@ -1654,7 +1606,7 @@
         <v>60.944699999999997</v>
       </c>
       <c r="G16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H16" s="2">
         <v>362194.35</v>
@@ -1674,22 +1626,19 @@
       <c r="M16" s="3">
         <v>45960</v>
       </c>
-      <c r="N16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
         <v>10</v>
-      </c>
-      <c r="C17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
       </c>
       <c r="E17">
         <v>873</v>
@@ -1698,7 +1647,7 @@
         <v>60.944699999999997</v>
       </c>
       <c r="G17" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H17" s="2">
         <v>53204.72</v>
@@ -1718,22 +1667,19 @@
       <c r="M17" s="3">
         <v>45960</v>
       </c>
-      <c r="N17" t="s">
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
       <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
         <v>10</v>
-      </c>
-      <c r="C18" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" t="s">
-        <v>12</v>
       </c>
       <c r="E18">
         <v>519</v>
@@ -1742,7 +1688,7 @@
         <v>60.944699999999997</v>
       </c>
       <c r="G18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H18" s="2">
         <v>31630.3</v>
@@ -1762,22 +1708,19 @@
       <c r="M18" s="3">
         <v>45960</v>
       </c>
-      <c r="N18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
         <v>9</v>
       </c>
-      <c r="B19" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" t="s">
-        <v>11</v>
-      </c>
       <c r="D19" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E19" s="1">
         <v>1200</v>
@@ -1786,7 +1729,7 @@
         <v>44.499600000000001</v>
       </c>
       <c r="G19" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H19" s="2">
         <v>53399.519999999997</v>
@@ -1805,9 +1748,6 @@
       </c>
       <c r="M19" s="3">
         <v>45960</v>
-      </c>
-      <c r="N19" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>